<commit_message>
Changed dependency for xver extensions
</commit_message>
<xml_diff>
--- a/models-src/oah-models-and-maps.xlsx
+++ b/models-src/oah-models-and-maps.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\oah\models-src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4561212D-6D29-488F-857E-9D760D31EABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9135FCD-67B7-48B8-A1E6-C0B0B9A70BE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-6510" yWindow="-21710" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{FA01C668-562A-4AF9-BDB0-B212F14DE883}"/>
+    <workbookView xWindow="-6510" yWindow="-21710" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{FA01C668-562A-4AF9-BDB0-B212F14DE883}"/>
   </bookViews>
   <sheets>
     <sheet name="ConceptMaps" sheetId="17" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1655" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1656" uniqueCount="565">
   <si>
     <t>Group Source</t>
   </si>
@@ -1751,6 +1751,9 @@
   </si>
   <si>
     <t>hospitalization.avoidablePrimaryPrevention</t>
+  </si>
+  <si>
+    <t>Hospitalizations</t>
   </si>
 </sst>
 </file>
@@ -1994,7 +1997,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2124,12 +2127,15 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -2156,6 +2162,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Hospital Discharge Report "/>
@@ -6913,9 +6920,9 @@
         <f>HealthIndicatorsOah!A57</f>
         <v>hospitalization</v>
       </c>
-      <c r="D57" s="8">
+      <c r="D57" s="8" t="str">
         <f>HealthIndicatorsOah!D57</f>
-        <v>0</v>
+        <v>Hospitalizations</v>
       </c>
       <c r="E57" s="8" t="s">
         <v>27</v>
@@ -8103,7 +8110,7 @@
         <v>522</v>
       </c>
       <c r="E52" s="59" t="str">
-        <f t="shared" ref="E52:E56" si="3">D52&amp;" - Cases per 100.000 inhabitants, per borough for each of the causes considered as relatable to the project"</f>
+        <f t="shared" ref="E52:E57" si="3">D52&amp;" - Cases per 100.000 inhabitants, per borough for each of the causes considered as relatable to the project"</f>
         <v>% of deaths due to cancer - Cases per 100.000 inhabitants, per borough for each of the causes considered as relatable to the project</v>
       </c>
     </row>
@@ -8180,7 +8187,7 @@
         <v>% of deaths due to COPD and lung cancer - Cases per 100.000 inhabitants, per borough for each of the causes considered as relatable to the project</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:6" ht="47.25" x14ac:dyDescent="0.45">
       <c r="A57" s="60" t="s">
         <v>554</v>
       </c>
@@ -8188,7 +8195,14 @@
         <v>14</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>485</v>
+        <v>29</v>
+      </c>
+      <c r="D57" s="63" t="s">
+        <v>564</v>
+      </c>
+      <c r="E57" s="59" t="str">
+        <f t="shared" si="3"/>
+        <v>Hospitalizations - Cases per 100.000 inhabitants, per borough for each of the causes considered as relatable to the project</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.45">

</xml_diff>